<commit_message>
Added tower guard to Gridmaze
</commit_message>
<xml_diff>
--- a/GridMaze/3_x_3_maze/3_x_3_maze_BOM.xlsx
+++ b/GridMaze/3_x_3_maze/3_x_3_maze_BOM.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60D2CA57-4E33-4493-B4D9-54656F0871CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{894073E0-0DAA-427D-939C-1A31C87515ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5490" yWindow="1110" windowWidth="16410" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="208">
   <si>
     <t>Part</t>
   </si>
@@ -617,6 +617,33 @@
   </si>
   <si>
     <t>1.5m</t>
+  </si>
+  <si>
+    <t>tower_guard</t>
+  </si>
+  <si>
+    <t>3D printed in ABS or PA12</t>
+  </si>
+  <si>
+    <t>Protolabs Network</t>
+  </si>
+  <si>
+    <t>tower_guard.stl</t>
+  </si>
+  <si>
+    <t>M3 x 12mm cap head screw</t>
+  </si>
+  <si>
+    <t>tower guard attachment</t>
+  </si>
+  <si>
+    <t>SCB3-12</t>
+  </si>
+  <si>
+    <t>Heat set thread insert M3</t>
+  </si>
+  <si>
+    <t>278-534</t>
   </si>
 </sst>
 </file>
@@ -1031,7 +1058,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I86"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
@@ -1322,49 +1349,46 @@
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>199</v>
+      </c>
+      <c r="B19" t="s">
+        <v>200</v>
+      </c>
+      <c r="C19">
+        <v>9</v>
+      </c>
+      <c r="D19" t="s">
+        <v>201</v>
+      </c>
+      <c r="E19" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="B20" s="1"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="1"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>2</v>
-      </c>
-      <c r="B21" t="s">
-        <v>159</v>
-      </c>
-      <c r="C21">
-        <v>9</v>
-      </c>
-      <c r="D21" t="s">
-        <v>7</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="I21" s="3"/>
+      <c r="B21" s="1"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="1"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>75</v>
+        <v>2</v>
       </c>
       <c r="B22" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C22">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D22" t="s">
         <v>7</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -1372,7 +1396,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>22</v>
+        <v>75</v>
       </c>
       <c r="B23" t="s">
         <v>160</v>
@@ -1384,7 +1408,7 @@
         <v>7</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>24</v>
+        <v>73</v>
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
@@ -1392,19 +1416,19 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="B24" t="s">
         <v>160</v>
       </c>
       <c r="C24">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D24" t="s">
         <v>7</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
@@ -1412,19 +1436,19 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>3</v>
+        <v>74</v>
       </c>
       <c r="B25" t="s">
         <v>160</v>
       </c>
       <c r="C25">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D25" t="s">
         <v>7</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
@@ -1432,19 +1456,19 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B26" t="s">
         <v>160</v>
       </c>
       <c r="C26">
+        <v>9</v>
+      </c>
+      <c r="D26" t="s">
+        <v>7</v>
+      </c>
+      <c r="E26" s="5" t="s">
         <v>4</v>
-      </c>
-      <c r="D26" t="s">
-        <v>7</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>174</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
@@ -1452,19 +1476,19 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>62</v>
+        <v>5</v>
       </c>
       <c r="B27" t="s">
         <v>160</v>
       </c>
       <c r="C27">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D27" t="s">
         <v>7</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
@@ -1472,10 +1496,10 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B28" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C28">
         <v>2</v>
@@ -1484,151 +1508,154 @@
         <v>7</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>120</v>
-      </c>
+        <v>175</v>
+      </c>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="I28" s="3"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>25</v>
+        <v>63</v>
       </c>
       <c r="B29" t="s">
-        <v>91</v>
+        <v>161</v>
       </c>
       <c r="C29">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D29" t="s">
         <v>7</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="F29" s="3"/>
-      <c r="G29" s="3"/>
-      <c r="I29" s="3"/>
+        <v>120</v>
+      </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B30" t="s">
-        <v>160</v>
+        <v>91</v>
       </c>
       <c r="C30">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="D30" t="s">
         <v>7</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>76</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="I30" s="3"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>117</v>
+        <v>26</v>
       </c>
       <c r="B31" t="s">
-        <v>119</v>
+        <v>160</v>
       </c>
       <c r="C31">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="D31" t="s">
         <v>7</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>118</v>
+        <v>76</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>176</v>
+        <v>117</v>
       </c>
       <c r="B32" t="s">
-        <v>162</v>
+        <v>119</v>
       </c>
       <c r="C32">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="D32" t="s">
-        <v>155</v>
-      </c>
-      <c r="E32" t="s">
-        <v>177</v>
+        <v>7</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>47</v>
+        <v>176</v>
       </c>
       <c r="B33" t="s">
-        <v>15</v>
+        <v>162</v>
       </c>
       <c r="C33">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D33" t="s">
-        <v>7</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>48</v>
+        <v>155</v>
+      </c>
+      <c r="E33" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="B34" t="s">
-        <v>186</v>
+        <v>15</v>
       </c>
       <c r="C34">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D34" t="s">
         <v>7</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="B35" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="C35">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="D35" t="s">
         <v>7</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B36" t="s">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="C36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D36" t="s">
         <v>7</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>9</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B37" t="s">
         <v>163</v>
@@ -1640,117 +1667,117 @@
         <v>7</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-      <c r="I37" s="3"/>
+        <v>9</v>
+      </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="B38" t="s">
-        <v>14</v>
+        <v>163</v>
       </c>
       <c r="C38">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D38" t="s">
         <v>7</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>11</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="I38" s="3"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="B39" t="s">
         <v>14</v>
       </c>
       <c r="C39">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="D39" t="s">
         <v>7</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>78</v>
+        <v>11</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="B40" t="s">
-        <v>179</v>
+        <v>14</v>
       </c>
       <c r="C40">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D40" t="s">
         <v>7</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>114</v>
+        <v>78</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>30</v>
+        <v>113</v>
       </c>
       <c r="B41" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C41">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D41" t="s">
         <v>7</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>79</v>
+        <v>114</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="B42" t="s">
-        <v>163</v>
+        <v>180</v>
       </c>
       <c r="C42">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D42" t="s">
         <v>7</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>12</v>
+        <v>79</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="B43" t="s">
         <v>163</v>
       </c>
       <c r="C43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D43" t="s">
         <v>7</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="B44" t="s">
         <v>163</v>
@@ -1762,29 +1789,32 @@
         <v>7</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B45" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="C45">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D45" t="s">
         <v>7</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>32</v>
+        <v>19</v>
+      </c>
+      <c r="B46" t="s">
+        <v>21</v>
       </c>
       <c r="C46">
         <v>4</v>
@@ -1793,15 +1823,12 @@
         <v>7</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>101</v>
+        <v>20</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>27</v>
-      </c>
-      <c r="B47" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C47">
         <v>4</v>
@@ -1810,29 +1837,29 @@
         <v>7</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>29</v>
+        <v>101</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B48" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="C48">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D48" t="s">
         <v>7</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B49" t="s">
         <v>35</v>
@@ -1841,30 +1868,27 @@
         <v>1</v>
       </c>
       <c r="D49" t="s">
-        <v>155</v>
-      </c>
-      <c r="E49" t="s">
-        <v>156</v>
-      </c>
-      <c r="F49" s="3"/>
-      <c r="G49" s="3"/>
-      <c r="I49" s="3"/>
+        <v>7</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>88</v>
+        <v>37</v>
       </c>
       <c r="B50" t="s">
-        <v>116</v>
+        <v>35</v>
       </c>
       <c r="C50">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="D50" t="s">
-        <v>7</v>
-      </c>
-      <c r="E50" s="5" t="s">
-        <v>90</v>
+        <v>155</v>
+      </c>
+      <c r="E50" t="s">
+        <v>156</v>
       </c>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
@@ -1872,19 +1896,19 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B51" t="s">
-        <v>187</v>
+        <v>116</v>
       </c>
       <c r="C51">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D51" t="s">
         <v>7</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
@@ -1892,19 +1916,19 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>158</v>
+        <v>93</v>
       </c>
       <c r="B52" t="s">
-        <v>86</v>
+        <v>187</v>
       </c>
       <c r="C52">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D52" t="s">
-        <v>57</v>
-      </c>
-      <c r="E52" s="5">
-        <v>2987669</v>
+        <v>7</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>92</v>
       </c>
       <c r="F52" s="3"/>
       <c r="G52" s="3"/>
@@ -1912,32 +1936,59 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>203</v>
       </c>
       <c r="B53" t="s">
-        <v>89</v>
+        <v>204</v>
       </c>
       <c r="C53">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D53" t="s">
-        <v>57</v>
-      </c>
-      <c r="E53" s="5">
-        <v>2987712</v>
+        <v>7</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>205</v>
       </c>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
       <c r="I53" s="3"/>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>158</v>
+      </c>
+      <c r="B54" t="s">
+        <v>86</v>
+      </c>
+      <c r="C54">
+        <v>18</v>
+      </c>
+      <c r="D54" t="s">
+        <v>57</v>
+      </c>
+      <c r="E54" s="5">
+        <v>2987669</v>
+      </c>
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
       <c r="I54" s="3"/>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
-        <v>84</v>
+      <c r="A55" t="s">
+        <v>103</v>
+      </c>
+      <c r="B55" t="s">
+        <v>89</v>
+      </c>
+      <c r="C55">
+        <v>4</v>
+      </c>
+      <c r="D55" t="s">
+        <v>57</v>
+      </c>
+      <c r="E55" s="5">
+        <v>2987712</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
@@ -1945,159 +1996,141 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>51</v>
+        <v>206</v>
+      </c>
+      <c r="B56" t="s">
+        <v>204</v>
       </c>
       <c r="C56">
         <v>9</v>
       </c>
       <c r="D56" t="s">
-        <v>50</v>
-      </c>
-      <c r="E56" s="5" t="s">
-        <v>194</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="E56" t="s">
+        <v>207</v>
+      </c>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
+      <c r="I56" s="3"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>52</v>
-      </c>
-      <c r="B57" t="s">
-        <v>195</v>
-      </c>
-      <c r="C57" t="s">
-        <v>196</v>
-      </c>
-      <c r="D57" t="s">
-        <v>148</v>
-      </c>
-      <c r="E57" t="s">
-        <v>149</v>
-      </c>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="I57" s="3"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>53</v>
-      </c>
-      <c r="B58" t="s">
-        <v>197</v>
-      </c>
-      <c r="C58" t="s">
-        <v>198</v>
-      </c>
-      <c r="D58" t="s">
-        <v>148</v>
-      </c>
-      <c r="E58" s="5" t="s">
-        <v>150</v>
-      </c>
+      <c r="A58" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
+      <c r="I58" s="3"/>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C59">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D59" t="s">
-        <v>148</v>
-      </c>
-      <c r="E59" t="s">
-        <v>151</v>
+        <v>50</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>55</v>
-      </c>
-      <c r="C60">
-        <v>9</v>
+        <v>52</v>
+      </c>
+      <c r="B60" t="s">
+        <v>195</v>
+      </c>
+      <c r="C60" t="s">
+        <v>196</v>
       </c>
       <c r="D60" t="s">
         <v>148</v>
       </c>
       <c r="E60" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>56</v>
-      </c>
-      <c r="C61">
-        <v>1</v>
+        <v>53</v>
+      </c>
+      <c r="B61" t="s">
+        <v>197</v>
+      </c>
+      <c r="C61" t="s">
+        <v>198</v>
       </c>
       <c r="D61" t="s">
         <v>148</v>
       </c>
-      <c r="E61" t="s">
-        <v>153</v>
+      <c r="E61" s="5" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>193</v>
-      </c>
-      <c r="E62"/>
+        <v>54</v>
+      </c>
+      <c r="C62">
+        <v>8</v>
+      </c>
+      <c r="D62" t="s">
+        <v>148</v>
+      </c>
+      <c r="E62" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>55</v>
+      </c>
+      <c r="C63">
+        <v>9</v>
+      </c>
+      <c r="D63" t="s">
+        <v>148</v>
+      </c>
+      <c r="E63" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A64" s="1" t="s">
-        <v>85</v>
+      <c r="A64" t="s">
+        <v>56</v>
+      </c>
+      <c r="C64">
+        <v>1</v>
+      </c>
+      <c r="D64" t="s">
+        <v>148</v>
+      </c>
+      <c r="E64" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>105</v>
-      </c>
-      <c r="B65" t="s">
-        <v>164</v>
-      </c>
-      <c r="C65">
-        <v>1</v>
-      </c>
-      <c r="D65" t="s">
-        <v>106</v>
-      </c>
-      <c r="E65" s="6" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>124</v>
-      </c>
-      <c r="B66" t="s">
-        <v>164</v>
-      </c>
-      <c r="C66">
-        <v>1</v>
-      </c>
-      <c r="D66" t="s">
-        <v>95</v>
-      </c>
-      <c r="E66" s="5" t="s">
-        <v>94</v>
-      </c>
+        <v>193</v>
+      </c>
+      <c r="E65"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>141</v>
-      </c>
-      <c r="B67" t="s">
-        <v>164</v>
-      </c>
-      <c r="C67">
-        <v>1</v>
-      </c>
-      <c r="D67" t="s">
-        <v>95</v>
-      </c>
-      <c r="E67" s="7" t="s">
-        <v>157</v>
+      <c r="A67" s="1" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>36</v>
+        <v>105</v>
       </c>
       <c r="B68" t="s">
         <v>164</v>
@@ -2106,18 +2139,18 @@
         <v>1</v>
       </c>
       <c r="D68" t="s">
-        <v>95</v>
-      </c>
-      <c r="E68" s="5" t="s">
-        <v>100</v>
+        <v>106</v>
+      </c>
+      <c r="E68" s="6" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>96</v>
+        <v>124</v>
       </c>
       <c r="B69" t="s">
-        <v>191</v>
+        <v>164</v>
       </c>
       <c r="C69">
         <v>1</v>
@@ -2126,15 +2159,15 @@
         <v>95</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>59</v>
+        <v>141</v>
       </c>
       <c r="B70" t="s">
-        <v>192</v>
+        <v>164</v>
       </c>
       <c r="C70">
         <v>1</v>
@@ -2142,135 +2175,135 @@
       <c r="D70" t="s">
         <v>95</v>
       </c>
-      <c r="E70" s="5" t="s">
-        <v>98</v>
+      <c r="E70" s="7" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>189</v>
+        <v>36</v>
       </c>
       <c r="B71" t="s">
-        <v>190</v>
+        <v>164</v>
       </c>
       <c r="C71">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D71" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>188</v>
+        <v>100</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="B72" t="s">
-        <v>107</v>
+        <v>191</v>
       </c>
       <c r="C72">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D72" t="s">
-        <v>57</v>
-      </c>
-      <c r="E72" s="5">
-        <v>1734905</v>
+        <v>95</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>109</v>
+        <v>59</v>
       </c>
       <c r="B73" t="s">
-        <v>107</v>
+        <v>192</v>
       </c>
       <c r="C73">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D73" t="s">
-        <v>57</v>
-      </c>
-      <c r="E73" s="5">
-        <v>1526172</v>
+        <v>95</v>
+      </c>
+      <c r="E73" s="5" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>108</v>
+        <v>189</v>
       </c>
       <c r="B74" t="s">
-        <v>107</v>
+        <v>190</v>
       </c>
       <c r="C74">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="D74" t="s">
-        <v>57</v>
-      </c>
-      <c r="E74" s="5">
-        <v>1734870</v>
+        <v>58</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>183</v>
+        <v>110</v>
       </c>
       <c r="B75" t="s">
-        <v>184</v>
+        <v>107</v>
       </c>
       <c r="C75">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D75" t="s">
         <v>57</v>
       </c>
       <c r="E75" s="5">
-        <v>4230976</v>
+        <v>1734905</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>185</v>
+        <v>109</v>
       </c>
       <c r="B76" t="s">
-        <v>184</v>
+        <v>107</v>
       </c>
       <c r="C76">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D76" t="s">
         <v>57</v>
       </c>
       <c r="E76" s="5">
-        <v>4230977</v>
+        <v>1526172</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B77" t="s">
-        <v>165</v>
+        <v>107</v>
       </c>
       <c r="C77">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D77" t="s">
         <v>57</v>
       </c>
       <c r="E77" s="5">
-        <v>2468268</v>
+        <v>1734870</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>112</v>
+        <v>183</v>
       </c>
       <c r="B78" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="C78">
         <v>1</v>
@@ -2279,95 +2312,146 @@
         <v>57</v>
       </c>
       <c r="E78" s="5">
-        <v>2646329</v>
+        <v>4230976</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>115</v>
+        <v>185</v>
       </c>
       <c r="B79" t="s">
-        <v>167</v>
+        <v>184</v>
       </c>
       <c r="C79">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D79" t="s">
         <v>57</v>
       </c>
       <c r="E79" s="5">
-        <v>1773450</v>
+        <v>4230977</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="B80" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C80">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="D80" t="s">
         <v>57</v>
       </c>
       <c r="E80" s="5">
-        <v>1416041</v>
+        <v>2468268</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>112</v>
+      </c>
+      <c r="B81" t="s">
+        <v>166</v>
+      </c>
+      <c r="C81">
+        <v>1</v>
+      </c>
+      <c r="D81" t="s">
+        <v>57</v>
+      </c>
+      <c r="E81" s="5">
+        <v>2646329</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" s="1" t="s">
-        <v>104</v>
+      <c r="A82" t="s">
+        <v>115</v>
+      </c>
+      <c r="B82" t="s">
+        <v>167</v>
+      </c>
+      <c r="C82">
+        <v>10</v>
+      </c>
+      <c r="D82" t="s">
+        <v>57</v>
+      </c>
+      <c r="E82" s="5">
+        <v>1773450</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>126</v>
+        <v>102</v>
+      </c>
+      <c r="B83" t="s">
+        <v>167</v>
       </c>
       <c r="C83">
-        <v>1</v>
-      </c>
-      <c r="E83" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>127</v>
-      </c>
-      <c r="C84">
-        <v>1</v>
-      </c>
-      <c r="E84" t="s">
-        <v>87</v>
+        <v>30</v>
+      </c>
+      <c r="D83" t="s">
+        <v>57</v>
+      </c>
+      <c r="E83" s="5">
+        <v>1416041</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>128</v>
-      </c>
-      <c r="C85">
-        <v>9</v>
-      </c>
-      <c r="E85" t="s">
-        <v>99</v>
+      <c r="A85" s="1" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>126</v>
+      </c>
+      <c r="C86">
+        <v>1</v>
+      </c>
+      <c r="E86" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>127</v>
+      </c>
+      <c r="C87">
+        <v>1</v>
+      </c>
+      <c r="E87" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>128</v>
+      </c>
+      <c r="C88">
+        <v>9</v>
+      </c>
+      <c r="E88" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>182</v>
       </c>
-      <c r="C86">
+      <c r="C89">
         <v>2</v>
       </c>
-      <c r="E86" t="s">
+      <c r="E89" t="s">
         <v>181</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E65" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="E68" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>

</xml_diff>